<commit_message>
write login page UI related test case
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9322A4C-E1CF-4F83-BB7C-5617E5A6646D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DAF9A7-4B89-4F2E-AD38-D1F5A796F966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Login" sheetId="1" r:id="rId1"/>
+    <sheet name="Login_page" sheetId="1" r:id="rId1"/>
     <sheet name="Products Page" sheetId="2" r:id="rId2"/>
     <sheet name="Product Shorting" sheetId="3" r:id="rId3"/>
     <sheet name="product Details" sheetId="4" r:id="rId4"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
   <si>
     <t>Test ID</t>
   </si>
@@ -87,13 +87,141 @@
   </si>
   <si>
     <t>Login page will loads successfully</t>
+  </si>
+  <si>
+    <t>TC_002</t>
+  </si>
+  <si>
+    <t>TC_003</t>
+  </si>
+  <si>
+    <t>TC_004</t>
+  </si>
+  <si>
+    <t>TC_005</t>
+  </si>
+  <si>
+    <t>TC_006</t>
+  </si>
+  <si>
+    <t>TC_007</t>
+  </si>
+  <si>
+    <t>TC_008</t>
+  </si>
+  <si>
+    <t>TC_009</t>
+  </si>
+  <si>
+    <t>TC_010</t>
+  </si>
+  <si>
+    <t>Verify application logo</t>
+  </si>
+  <si>
+    <t>Open Login page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logo will visible </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Logo is visible </t>
+  </si>
+  <si>
+    <t>Verify username field</t>
+  </si>
+  <si>
+    <t>Username is visible and enable</t>
+  </si>
+  <si>
+    <t>Verify password field</t>
+  </si>
+  <si>
+    <t>Username field will visible and enable</t>
+  </si>
+  <si>
+    <t>Password field will visible and enable</t>
+  </si>
+  <si>
+    <t>Password fiels is visible and enable</t>
+  </si>
+  <si>
+    <t>Verify Login Button</t>
+  </si>
+  <si>
+    <t>Test Step</t>
+  </si>
+  <si>
+    <t>Login button will visible and clickable</t>
+  </si>
+  <si>
+    <t>Login button is visble and clickable</t>
+  </si>
+  <si>
+    <t>Verify password masking</t>
+  </si>
+  <si>
+    <t>Enter a password</t>
+  </si>
+  <si>
+    <t>Password will be making</t>
+  </si>
+  <si>
+    <t>passwod is masking.</t>
+  </si>
+  <si>
+    <t>Verify username placeholder</t>
+  </si>
+  <si>
+    <t>Corrent username placeholde will be
+display.</t>
+  </si>
+  <si>
+    <t>Correct username is displayed</t>
+  </si>
+  <si>
+    <t>Verify password placeholder</t>
+  </si>
+  <si>
+    <t>Corrent Password placeholde will be
+display.</t>
+  </si>
+  <si>
+    <t>Correct password is displayed</t>
+  </si>
+  <si>
+    <t>Verify keyboard tab order</t>
+  </si>
+  <si>
+    <t>Press tab repeatedly</t>
+  </si>
+  <si>
+    <t>Press Tab key</t>
+  </si>
+  <si>
+    <t>Focus moves logically through controls</t>
+  </si>
+  <si>
+    <t>Moves successfully after press tab</t>
+  </si>
+  <si>
+    <t>Verify Enter key login</t>
+  </si>
+  <si>
+    <t>Press Enter key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User will loged in successfully after pressEnter key. </t>
+  </si>
+  <si>
+    <t>User Login successfully.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,6 +230,19 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -128,10 +269,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -414,41 +561,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B8:I9"/>
+  <dimension ref="B8:I18"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
     <col min="3" max="3" width="42.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="36.85546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="18.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="30.42578125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28" style="1" customWidth="1"/>
+    <col min="6" max="6" width="35.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="8" spans="2:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="2" t="s">
+    <row r="8" spans="2:9" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D8" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E8" s="2" t="s">
+      <c r="D8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="I8" s="4" t="s">
         <v>7</v>
       </c>
     </row>
@@ -478,7 +625,242 @@
         <v>15</v>
       </c>
     </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E14" s="1">
+        <v>12344555</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B17" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B18" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="3" t="s">
+        <v>57</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9:H30" xr:uid="{BB47CFD5-A71F-4422-A100-436DB6CAFF84}">
       <formula1>"Criticale, High, Medium, Low"</formula1>
@@ -488,6 +870,7 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
write login positive test case
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2DAF9A7-4B89-4F2E-AD38-D1F5A796F966}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3532D730-34C3-4B92-A12D-ED8C8B8421F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="80">
   <si>
     <t>Test ID</t>
   </si>
@@ -215,6 +215,72 @@
   </si>
   <si>
     <t>User Login successfully.</t>
+  </si>
+  <si>
+    <t>TC_011</t>
+  </si>
+  <si>
+    <t>TC_012</t>
+  </si>
+  <si>
+    <t>TC_013</t>
+  </si>
+  <si>
+    <t>TC_014</t>
+  </si>
+  <si>
+    <t>TC_015</t>
+  </si>
+  <si>
+    <t>Verify Login with standard User</t>
+  </si>
+  <si>
+    <t>Enter Valid data</t>
+  </si>
+  <si>
+    <t>standard_user /
+secret_sauce</t>
+  </si>
+  <si>
+    <t>Login successfully</t>
+  </si>
+  <si>
+    <t>Login with Problem user</t>
+  </si>
+  <si>
+    <t>Enter problem user data</t>
+  </si>
+  <si>
+    <t>problem_user / 
+secret_sauce</t>
+  </si>
+  <si>
+    <t>Login with performance user</t>
+  </si>
+  <si>
+    <t>Enter performance user data</t>
+  </si>
+  <si>
+    <t>Login with error User</t>
+  </si>
+  <si>
+    <t>Enter error user data</t>
+  </si>
+  <si>
+    <t>error_user / secret_sauce</t>
+  </si>
+  <si>
+    <t>performance_glitch_user/
+secret_sauce</t>
+  </si>
+  <si>
+    <t>Login with visula user</t>
+  </si>
+  <si>
+    <t>Enter Visul user data</t>
+  </si>
+  <si>
+    <t>visula_user / secret_sauce</t>
   </si>
 </sst>
 </file>
@@ -269,7 +335,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -280,6 +346,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -561,13 +630,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B8:I18"/>
+  <dimension ref="B8:I23"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
     <col min="3" max="3" width="42.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="36.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="18.140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="35.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
@@ -859,13 +928,143 @@
         <v>15</v>
       </c>
     </row>
+    <row r="19" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B19" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B20" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I20" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="2:9" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="B21" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>76</v>
+      </c>
+      <c r="F21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B22" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B23" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9:H30" xr:uid="{BB47CFD5-A71F-4422-A100-436DB6CAFF84}">
       <formula1>"Criticale, High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I9:I22" xr:uid="{C9603965-C732-484C-98AF-3D6F90CB9B65}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I9:I23" xr:uid="{C9603965-C732-484C-98AF-3D6F90CB9B65}">
       <formula1>"Passed, Failed, Skipped, Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
write negative test case for login form
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3532D730-34C3-4B92-A12D-ED8C8B8421F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D24C687-3409-4EE6-97A8-CC79195178C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="150">
   <si>
     <t>Test ID</t>
   </si>
@@ -245,9 +245,6 @@
     <t>Login successfully</t>
   </si>
   <si>
-    <t>Login with Problem user</t>
-  </si>
-  <si>
     <t>Enter problem user data</t>
   </si>
   <si>
@@ -255,13 +252,7 @@
 secret_sauce</t>
   </si>
   <si>
-    <t>Login with performance user</t>
-  </si>
-  <si>
     <t>Enter performance user data</t>
-  </si>
-  <si>
-    <t>Login with error User</t>
   </si>
   <si>
     <t>Enter error user data</t>
@@ -274,13 +265,234 @@
 secret_sauce</t>
   </si>
   <si>
-    <t>Login with visula user</t>
-  </si>
-  <si>
     <t>Enter Visul user data</t>
   </si>
   <si>
     <t>visula_user / secret_sauce</t>
+  </si>
+  <si>
+    <t>TC_016</t>
+  </si>
+  <si>
+    <t>TC_017</t>
+  </si>
+  <si>
+    <t>TC_018</t>
+  </si>
+  <si>
+    <t>TC_019</t>
+  </si>
+  <si>
+    <t>TC_020</t>
+  </si>
+  <si>
+    <t>TC_021</t>
+  </si>
+  <si>
+    <t>TC_022</t>
+  </si>
+  <si>
+    <t>TC_023</t>
+  </si>
+  <si>
+    <t>TC_024</t>
+  </si>
+  <si>
+    <t>TC_025</t>
+  </si>
+  <si>
+    <t>TC_026</t>
+  </si>
+  <si>
+    <t>TC_027</t>
+  </si>
+  <si>
+    <t>TC_028</t>
+  </si>
+  <si>
+    <t>TC_029</t>
+  </si>
+  <si>
+    <t>TC_030</t>
+  </si>
+  <si>
+    <t>TC_031</t>
+  </si>
+  <si>
+    <t>TC_032</t>
+  </si>
+  <si>
+    <t>Enter a Invalid user</t>
+  </si>
+  <si>
+    <t>Invalid user / secret_sauce</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login will blocked with a error message </t>
+  </si>
+  <si>
+    <t>Login is blocked and show a 
+error message.</t>
+  </si>
+  <si>
+    <t>Enter a invalid password</t>
+  </si>
+  <si>
+    <t>standard_user /
+invalid_password</t>
+  </si>
+  <si>
+    <t>Enter a invalid user &amp; invalid password</t>
+  </si>
+  <si>
+    <t>Invalid user / invalid password</t>
+  </si>
+  <si>
+    <t>Verify Login with Problem user</t>
+  </si>
+  <si>
+    <t>Verify Login with performance user</t>
+  </si>
+  <si>
+    <t>Verify Login with error User</t>
+  </si>
+  <si>
+    <t>Verify Login with visula user</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid user</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid password</t>
+  </si>
+  <si>
+    <t>Verify Login with Invalid user &amp; invalid password</t>
+  </si>
+  <si>
+    <t>Verify Login with empty username</t>
+  </si>
+  <si>
+    <t>Enter empty user &amp; valid password</t>
+  </si>
+  <si>
+    <t>Blank username / valid password</t>
+  </si>
+  <si>
+    <t>Verify Login with empty password</t>
+  </si>
+  <si>
+    <t>Enter valid user &amp; empty password</t>
+  </si>
+  <si>
+    <t>valid username / blank password</t>
+  </si>
+  <si>
+    <t>Enter both empty field</t>
+  </si>
+  <si>
+    <t>Blank field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verigy Login with locked out user </t>
+  </si>
+  <si>
+    <t>Verify Login both field empty</t>
+  </si>
+  <si>
+    <t>Enter locked out user data</t>
+  </si>
+  <si>
+    <t>locked out user / secret_sauce</t>
+  </si>
+  <si>
+    <t>Enter user name with leding space</t>
+  </si>
+  <si>
+    <t>standard_user</t>
+  </si>
+  <si>
+    <t>Enter user name with agfter space</t>
+  </si>
+  <si>
+    <t>Verify login with leading space username</t>
+  </si>
+  <si>
+    <t>Verify login with after spaceusername</t>
+  </si>
+  <si>
+    <t>Verify login with leading space password</t>
+  </si>
+  <si>
+    <t>Enter password with leading space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  secret_sauce</t>
+  </si>
+  <si>
+    <t>Verify login with after space password</t>
+  </si>
+  <si>
+    <t>Enter password with after space</t>
+  </si>
+  <si>
+    <t xml:space="preserve">secret_sauce   </t>
+  </si>
+  <si>
+    <t>Verify login with username case sensitivity</t>
+  </si>
+  <si>
+    <t>Enter user name with case sensitivity</t>
+  </si>
+  <si>
+    <t>STANDARD_USER</t>
+  </si>
+  <si>
+    <t>Verigy Login with password case sensitivity</t>
+  </si>
+  <si>
+    <t>Enter password case sensitivity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECRET_SAUCE   </t>
+  </si>
+  <si>
+    <t>Enter a long user name</t>
+  </si>
+  <si>
+    <t>30+ characters</t>
+  </si>
+  <si>
+    <t>Enter a long password</t>
+  </si>
+  <si>
+    <t>40+ characters</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify with login username </t>
+  </si>
+  <si>
+    <t>Verify with login password</t>
+  </si>
+  <si>
+    <t>Verify with login special character in Username</t>
+  </si>
+  <si>
+    <t>Enter special character in username</t>
+  </si>
+  <si>
+    <t>(**&amp;%&amp;$^%</t>
+  </si>
+  <si>
+    <t>Verify multiple faild login attempts</t>
+  </si>
+  <si>
+    <t>Enter invalid data repetedly</t>
+  </si>
+  <si>
+    <t>Multiple time try with invalid data</t>
+  </si>
+  <si>
+    <t>Application handles attempts correctly</t>
   </si>
 </sst>
 </file>
@@ -335,7 +547,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -346,9 +558,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -630,15 +839,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B8:I23"/>
+  <dimension ref="B8:I45"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="9.140625" style="1"/>
     <col min="3" max="3" width="42.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="36.85546875" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="35.140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.7109375" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
@@ -669,158 +878,158 @@
       </c>
     </row>
     <row r="9" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F9" s="1" t="s">
+      <c r="F9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I9" s="1" t="s">
+      <c r="H9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I9" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="1" t="s">
+      <c r="F10" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="H10" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I10" s="1" t="s">
+      <c r="H10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="F11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="H11" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I11" s="1" t="s">
+      <c r="H11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I11" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="12" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F12" s="1" t="s">
+      <c r="F12" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I12" s="1" t="s">
+      <c r="H12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I12" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="F13" s="1" t="s">
+      <c r="F13" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="H13" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I13" s="1" t="s">
+      <c r="H13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I13" s="2" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D14" s="1" t="s">
+      <c r="D14" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="2">
         <v>12344555</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F14" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="H14" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I14" s="1" t="s">
+      <c r="H14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -877,28 +1086,28 @@
       </c>
     </row>
     <row r="17" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="D17" s="1" t="s">
+      <c r="D17" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F17" s="1" t="s">
+      <c r="F17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="H17" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I17" s="1" t="s">
+      <c r="H17" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -932,25 +1141,25 @@
       <c r="B19" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="D19" s="1" t="s">
+      <c r="D19" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="E19" s="5" t="s">
+      <c r="E19" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="F19" s="1" t="s">
+      <c r="F19" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="H19" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I19" s="1" t="s">
+      <c r="H19" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I19" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -959,13 +1168,13 @@
         <v>60</v>
       </c>
       <c r="C20" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="E20" s="3" t="s">
         <v>69</v>
-      </c>
-      <c r="E20" s="3" t="s">
-        <v>70</v>
       </c>
       <c r="F20" s="2" t="s">
         <v>67</v>
@@ -980,18 +1189,18 @@
         <v>15</v>
       </c>
     </row>
-    <row r="21" spans="2:9" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
         <v>61</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>71</v>
+        <v>102</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>67</v>
@@ -1010,25 +1219,25 @@
       <c r="B22" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D22" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E22" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F22" s="1" t="s">
+      <c r="C22" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D22" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="F22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="G22" s="1" t="s">
+      <c r="G22" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="H22" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I22" s="1" t="s">
+      <c r="H22" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1036,35 +1245,522 @@
       <c r="B23" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C23" s="1" t="s">
+      <c r="C23" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="F23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B24" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D24" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F24" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G24" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B25" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="C25" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="E25" s="3" t="s">
+        <v>98</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G25" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B26" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E23" s="1" t="s">
+      <c r="C26" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G26" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="27" spans="2:9" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B27" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F23" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="G23" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I23" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="C27" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="28" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="D28" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="29" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B29" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G29" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="30" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B30" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>118</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="F30" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G30" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="31" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B31" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F31" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="F32" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G32" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B33" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="F33" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G33" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B34" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="F34" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G34" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B35" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="E35" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G35" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B36" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G36" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B37" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G37" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I37" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>139</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G38" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G39" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B40" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="41" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B41" s="2"/>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2"/>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B42" s="2"/>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B43" s="2"/>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2"/>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
+      <c r="H45" s="2"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9:H30" xr:uid="{BB47CFD5-A71F-4422-A100-436DB6CAFF84}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H9:H40" xr:uid="{BB47CFD5-A71F-4422-A100-436DB6CAFF84}">
       <formula1>"Criticale, High, Medium, Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I9:I23" xr:uid="{C9603965-C732-484C-98AF-3D6F90CB9B65}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I9:I40" xr:uid="{C9603965-C732-484C-98AF-3D6F90CB9B65}">
       <formula1>"Passed, Failed, Skipped, Blocked"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
write test case for products page UI test
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D24C687-3409-4EE6-97A8-CC79195178C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C037A12-132A-47CF-B7EA-E9DD5BFDF135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="272" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="191">
   <si>
     <t>Test ID</t>
   </si>
@@ -493,6 +493,130 @@
   </si>
   <si>
     <t>Application handles attempts correctly</t>
+  </si>
+  <si>
+    <t>Verify product page after login</t>
+  </si>
+  <si>
+    <t>View product page after login</t>
+  </si>
+  <si>
+    <t>Should be logedin</t>
+  </si>
+  <si>
+    <t>Product page will view after login</t>
+  </si>
+  <si>
+    <t>Product page is login after login</t>
+  </si>
+  <si>
+    <t>Pass</t>
+  </si>
+  <si>
+    <t>Verify the page title</t>
+  </si>
+  <si>
+    <t>View the correct page title</t>
+  </si>
+  <si>
+    <t>Page title will be display</t>
+  </si>
+  <si>
+    <t>Page title is display</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Verify all product are display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View the all products </t>
+  </si>
+  <si>
+    <t>All products will be display</t>
+  </si>
+  <si>
+    <t>All products displayed</t>
+  </si>
+  <si>
+    <t>Verify each product image visible</t>
+  </si>
+  <si>
+    <t>View each product image</t>
+  </si>
+  <si>
+    <t>Each product image is visible</t>
+  </si>
+  <si>
+    <t>Verify each product name</t>
+  </si>
+  <si>
+    <t>Product name is displayed</t>
+  </si>
+  <si>
+    <t>Verify product description</t>
+  </si>
+  <si>
+    <t>Product description is displayed</t>
+  </si>
+  <si>
+    <t>Verify product price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">View product name </t>
+  </si>
+  <si>
+    <t>View product description</t>
+  </si>
+  <si>
+    <t>View product price</t>
+  </si>
+  <si>
+    <t>Product is displayed</t>
+  </si>
+  <si>
+    <t>Verify add to cart button</t>
+  </si>
+  <si>
+    <t>View add to cart product</t>
+  </si>
+  <si>
+    <t>Add to cart button is displayed for all products</t>
+  </si>
+  <si>
+    <t>Verify product container layout</t>
+  </si>
+  <si>
+    <t>Check the prodcut container</t>
+  </si>
+  <si>
+    <t>Product display without overlap</t>
+  </si>
+  <si>
+    <t>Verify product details navigation</t>
+  </si>
+  <si>
+    <t>Check the product details navigation</t>
+  </si>
+  <si>
+    <t>Navigate to the product details page</t>
+  </si>
+  <si>
+    <t>Navigation faile, not navigate</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Failed</t>
+  </si>
+  <si>
+    <t>Verify product image navigation</t>
+  </si>
+  <si>
+    <t>Check the product image click
+ navigation</t>
   </si>
 </sst>
 </file>
@@ -1798,39 +1922,401 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{592A122A-5D5B-4999-ABE1-908A0253B8D0}">
-  <dimension ref="B5:J5"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="B5:J19"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="2" width="9.140625" style="1"/>
+    <col min="3" max="3" width="30.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="5" spans="2:10" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B5" s="1" t="s">
+    <row r="5" spans="2:10" s="4" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="F5" s="1" t="s">
+      <c r="F5" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H5" s="1" t="s">
+      <c r="H5" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="I5" s="1" t="s">
+      <c r="I5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="J5" s="1" t="s">
+      <c r="J5" s="4" t="s">
         <v>7</v>
       </c>
     </row>
+    <row r="6" spans="2:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B8" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B9" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B13" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>179</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>160</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B15" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="H15" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" s="2" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>185</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I6:I19" xr:uid="{43B99713-1CFD-494D-B744-65C2C2E214D0}">
+      <formula1>"Cirticale, High,Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J16:J19" xr:uid="{A51009FC-9E19-41F9-9266-C3C78A4FF497}">
+      <formula1>"Pass, Faild, Skip, Block"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J6:J15" xr:uid="{C6D868CF-0C39-47E8-A6C8-2A3C81D619ED}">
+      <formula1>"Passed, Failed, Blocked, Skip"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test cases for product page
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C037A12-132A-47CF-B7EA-E9DD5BFDF135}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02FC48D8-CC3B-4828-92A6-5E846F9B0064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="239">
   <si>
     <t>Test ID</t>
   </si>
@@ -617,6 +617,161 @@
   <si>
     <t>Check the product image click
  navigation</t>
+  </si>
+  <si>
+    <t>Verify sort dropdown visibility</t>
+  </si>
+  <si>
+    <t>Check the sort dropdown visible.</t>
+  </si>
+  <si>
+    <t>The product sort dropdown will be visible</t>
+  </si>
+  <si>
+    <t>The product dropdown is visible</t>
+  </si>
+  <si>
+    <t>Verify sort name A to Z</t>
+  </si>
+  <si>
+    <t>Check the sort name A to Z</t>
+  </si>
+  <si>
+    <t>Must be login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product sort A to Z will be in the dropdown. </t>
+  </si>
+  <si>
+    <t>Pordut short A to Z in the dropdown</t>
+  </si>
+  <si>
+    <t>Verify sort name Z to A</t>
+  </si>
+  <si>
+    <t>Check the sort name Z to A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Product sort Z to A will be in the dropdown. </t>
+  </si>
+  <si>
+    <t>Pordut short Z to A in the dropdown</t>
+  </si>
+  <si>
+    <t>Verify sort price Low to High</t>
+  </si>
+  <si>
+    <t>Check sort price Low to High</t>
+  </si>
+  <si>
+    <t>Product sort price low to high will be in 
+the dropdown</t>
+  </si>
+  <si>
+    <t>Product sort price low to high in the
+ dropdown</t>
+  </si>
+  <si>
+    <t>Verify sort price High to Low</t>
+  </si>
+  <si>
+    <t>Check sort price High to Low</t>
+  </si>
+  <si>
+    <t>Product sort price High to Low will be in 
+the dropdown</t>
+  </si>
+  <si>
+    <t>Product sort price High to Low in the
+ dropdown</t>
+  </si>
+  <si>
+    <t>Verify default sorting</t>
+  </si>
+  <si>
+    <t>Check the default sorting</t>
+  </si>
+  <si>
+    <t>Default sorting is correct</t>
+  </si>
+  <si>
+    <t>Verfy sorting multiple time</t>
+  </si>
+  <si>
+    <t>Check sorting multiple time</t>
+  </si>
+  <si>
+    <t>Product sort update each time perfectly</t>
+  </si>
+  <si>
+    <t>Verify add product after sorting</t>
+  </si>
+  <si>
+    <t>Check add product after sort</t>
+  </si>
+  <si>
+    <t>Correct product is added after sort</t>
+  </si>
+  <si>
+    <t>Verify with items already in cart</t>
+  </si>
+  <si>
+    <t>Check item already in the cart</t>
+  </si>
+  <si>
+    <t>Cart content remain unchange</t>
+  </si>
+  <si>
+    <t>Verify Refresh after sorting</t>
+  </si>
+  <si>
+    <t>Check refresh after sort</t>
+  </si>
+  <si>
+    <t>Sorting product will not be change</t>
+  </si>
+  <si>
+    <t>shorting data change after refresh</t>
+  </si>
+  <si>
+    <t>Verify sort dropdown keyboard
+access</t>
+  </si>
+  <si>
+    <t>Check the dropdown keyboard 
+access</t>
+  </si>
+  <si>
+    <t>Dropdwon menu can be operate from keyboard</t>
+  </si>
+  <si>
+    <t>Dropdown menu operate from the 
+keyboard</t>
+  </si>
+  <si>
+    <t>Verify no duplicate product after sorting.</t>
+  </si>
+  <si>
+    <t>Check duplicater product after
+ sorting</t>
+  </si>
+  <si>
+    <t>Duplicate product is appears after sorting</t>
+  </si>
+  <si>
+    <t>No duplicate product is appears
+ after sorting</t>
+  </si>
+  <si>
+    <t>Verify prices remain associated 
+with correct products</t>
+  </si>
+  <si>
+    <t>Checke the prices with the Correct
+Product.</t>
+  </si>
+  <si>
+    <t>Product price remains consistent</t>
   </si>
 </sst>
 </file>
@@ -671,7 +826,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -682,6 +837,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2323,9 +2481,434 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{330326CC-6D37-4000-8F1B-014F814374DB}">
-  <dimension ref="A1"/>
+  <dimension ref="B4:J17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="3" max="3" width="29.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="30.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="43.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="2:10" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="B4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>191</v>
+      </c>
+      <c r="D5" t="s">
+        <v>192</v>
+      </c>
+      <c r="E5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F5" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" t="s">
+        <v>193</v>
+      </c>
+      <c r="H5" t="s">
+        <v>194</v>
+      </c>
+      <c r="I5" t="s">
+        <v>14</v>
+      </c>
+      <c r="J5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" t="s">
+        <v>195</v>
+      </c>
+      <c r="D6" t="s">
+        <v>196</v>
+      </c>
+      <c r="E6" t="s">
+        <v>197</v>
+      </c>
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>198</v>
+      </c>
+      <c r="H6" t="s">
+        <v>199</v>
+      </c>
+      <c r="I6" t="s">
+        <v>14</v>
+      </c>
+      <c r="J6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D7" t="s">
+        <v>201</v>
+      </c>
+      <c r="E7" t="s">
+        <v>197</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>202</v>
+      </c>
+      <c r="H7" t="s">
+        <v>203</v>
+      </c>
+      <c r="I7" t="s">
+        <v>14</v>
+      </c>
+      <c r="J7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D8" t="s">
+        <v>205</v>
+      </c>
+      <c r="E8" t="s">
+        <v>197</v>
+      </c>
+      <c r="F8" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="H8" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="I8" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>20</v>
+      </c>
+      <c r="C9" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" t="s">
+        <v>209</v>
+      </c>
+      <c r="E9" t="s">
+        <v>197</v>
+      </c>
+      <c r="F9" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="I9" t="s">
+        <v>14</v>
+      </c>
+      <c r="J9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C10" t="s">
+        <v>212</v>
+      </c>
+      <c r="D10" t="s">
+        <v>213</v>
+      </c>
+      <c r="E10" t="s">
+        <v>197</v>
+      </c>
+      <c r="F10" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" t="s">
+        <v>214</v>
+      </c>
+      <c r="H10" t="s">
+        <v>214</v>
+      </c>
+      <c r="I10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s">
+        <v>215</v>
+      </c>
+      <c r="D11" t="s">
+        <v>216</v>
+      </c>
+      <c r="E11" t="s">
+        <v>197</v>
+      </c>
+      <c r="F11" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" t="s">
+        <v>217</v>
+      </c>
+      <c r="H11" t="s">
+        <v>217</v>
+      </c>
+      <c r="I11" t="s">
+        <v>14</v>
+      </c>
+      <c r="J11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" t="s">
+        <v>23</v>
+      </c>
+      <c r="C12" t="s">
+        <v>218</v>
+      </c>
+      <c r="D12" t="s">
+        <v>219</v>
+      </c>
+      <c r="E12" t="s">
+        <v>197</v>
+      </c>
+      <c r="F12" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" t="s">
+        <v>220</v>
+      </c>
+      <c r="H12" t="s">
+        <v>220</v>
+      </c>
+      <c r="I12" t="s">
+        <v>14</v>
+      </c>
+      <c r="J12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B13" t="s">
+        <v>24</v>
+      </c>
+      <c r="C13" t="s">
+        <v>221</v>
+      </c>
+      <c r="D13" t="s">
+        <v>222</v>
+      </c>
+      <c r="E13" t="s">
+        <v>197</v>
+      </c>
+      <c r="F13" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" t="s">
+        <v>223</v>
+      </c>
+      <c r="H13" t="s">
+        <v>223</v>
+      </c>
+      <c r="I13" t="s">
+        <v>14</v>
+      </c>
+      <c r="J13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B14" t="s">
+        <v>25</v>
+      </c>
+      <c r="C14" t="s">
+        <v>224</v>
+      </c>
+      <c r="D14" t="s">
+        <v>225</v>
+      </c>
+      <c r="E14" t="s">
+        <v>197</v>
+      </c>
+      <c r="F14" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" t="s">
+        <v>226</v>
+      </c>
+      <c r="H14" t="s">
+        <v>227</v>
+      </c>
+      <c r="I14" t="s">
+        <v>14</v>
+      </c>
+      <c r="J14" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B15" t="s">
+        <v>59</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="E15" t="s">
+        <v>197</v>
+      </c>
+      <c r="F15" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" t="s">
+        <v>230</v>
+      </c>
+      <c r="H15" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="I15" t="s">
+        <v>14</v>
+      </c>
+      <c r="J15" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B16" t="s">
+        <v>60</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>233</v>
+      </c>
+      <c r="E16" t="s">
+        <v>197</v>
+      </c>
+      <c r="F16" t="s">
+        <v>12</v>
+      </c>
+      <c r="G16" t="s">
+        <v>234</v>
+      </c>
+      <c r="H16" s="5" t="s">
+        <v>235</v>
+      </c>
+      <c r="I16" t="s">
+        <v>14</v>
+      </c>
+      <c r="J16" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>236</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>237</v>
+      </c>
+      <c r="E17" t="s">
+        <v>197</v>
+      </c>
+      <c r="F17" t="s">
+        <v>12</v>
+      </c>
+      <c r="G17" t="s">
+        <v>238</v>
+      </c>
+      <c r="H17" t="s">
+        <v>238</v>
+      </c>
+      <c r="I17" t="s">
+        <v>14</v>
+      </c>
+      <c r="J17" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I5:I17" xr:uid="{E50581E8-E171-4FF5-8858-A19175C29410}">
+      <formula1>"Critcal, High, Medium, Low"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J5:J17" xr:uid="{66484086-A554-4DEB-9033-F8C51B4534CD}">
+      <formula1>"Passed, Blodked, Failed, Skiped"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test cases for add to cart
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02FC48D8-CC3B-4828-92A6-5E846F9B0064}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8212CC8-44D8-4AAC-8724-696871B4309B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="306">
   <si>
     <t>Test ID</t>
   </si>
@@ -772,6 +772,222 @@
   </si>
   <si>
     <t>Product price remains consistent</t>
+  </si>
+  <si>
+    <t>Verify open product details page using
+name</t>
+  </si>
+  <si>
+    <t>Check the product details page using
+name</t>
+  </si>
+  <si>
+    <t>Correct product details page 
+is open</t>
+  </si>
+  <si>
+    <t>Verify open product details page using
+image</t>
+  </si>
+  <si>
+    <t>Check the product details page using
+image</t>
+  </si>
+  <si>
+    <t>Verify selected product name</t>
+  </si>
+  <si>
+    <t>Verify selected product image</t>
+  </si>
+  <si>
+    <t>Check the product details page match 
+the product name.</t>
+  </si>
+  <si>
+    <t>Check the product details page match 
+the product image.</t>
+  </si>
+  <si>
+    <t>Match the selected product name</t>
+  </si>
+  <si>
+    <t>Display the slected product image</t>
+  </si>
+  <si>
+    <t>Verify the product description</t>
+  </si>
+  <si>
+    <t>Correct description is display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check the product description </t>
+  </si>
+  <si>
+    <t>Check the product price</t>
+  </si>
+  <si>
+    <t>Display the correct price</t>
+  </si>
+  <si>
+    <t>Checke add product from details page</t>
+  </si>
+  <si>
+    <t>Add product successfully</t>
+  </si>
+  <si>
+    <t>Verify add to cart product from
+ details page</t>
+  </si>
+  <si>
+    <t>Verify remove from cart product 
+from details page</t>
+  </si>
+  <si>
+    <t>Check remove product from cart</t>
+  </si>
+  <si>
+    <t>Remove product from cart</t>
+  </si>
+  <si>
+    <t>Verify cart dadge after adding</t>
+  </si>
+  <si>
+    <t>Check the cart badge after add product</t>
+  </si>
+  <si>
+    <t>Cart badge will show after add
+ product</t>
+  </si>
+  <si>
+    <t>Cart badge is show after add
+ product</t>
+  </si>
+  <si>
+    <t>Verify Back to product button</t>
+  </si>
+  <si>
+    <t>Check Back to product button</t>
+  </si>
+  <si>
+    <t>Back to the product page by clicking
+Back to products button</t>
+  </si>
+  <si>
+    <t>Verify product remains in cart after 
+returning</t>
+  </si>
+  <si>
+    <t>Cart sate is preserved</t>
+  </si>
+  <si>
+    <t>Verify refresh details page</t>
+  </si>
+  <si>
+    <t>Check product is preserved</t>
+  </si>
+  <si>
+    <t>Check product refresh after refresh</t>
+  </si>
+  <si>
+    <t>Product details is correct after 
+refresh</t>
+  </si>
+  <si>
+    <t>Checke add a product</t>
+  </si>
+  <si>
+    <t>Product added</t>
+  </si>
+  <si>
+    <t>The product added</t>
+  </si>
+  <si>
+    <t>Verify add one product</t>
+  </si>
+  <si>
+    <t>Verify add multiple product</t>
+  </si>
+  <si>
+    <t>Check add multiple product</t>
+  </si>
+  <si>
+    <t>All  selected product added</t>
+  </si>
+  <si>
+    <t>Verify add all availale products</t>
+  </si>
+  <si>
+    <t>All available product added correctly</t>
+  </si>
+  <si>
+    <t>Verify cart badge after add item</t>
+  </si>
+  <si>
+    <t>Check add all available products</t>
+  </si>
+  <si>
+    <t>Check the card badge</t>
+  </si>
+  <si>
+    <t>Cart badge is show</t>
+  </si>
+  <si>
+    <t>Verify add product twice rapidly</t>
+  </si>
+  <si>
+    <t>Check add twice rapidly</t>
+  </si>
+  <si>
+    <t>Product is not duplicate unexpectedly</t>
+  </si>
+  <si>
+    <t>Verify add item from product details</t>
+  </si>
+  <si>
+    <t>Check add product from product details</t>
+  </si>
+  <si>
+    <t>Cart update correctly</t>
+  </si>
+  <si>
+    <t>Verify add item after sorting</t>
+  </si>
+  <si>
+    <t>Check add item after sorting</t>
+  </si>
+  <si>
+    <t>Correct item will be added</t>
+  </si>
+  <si>
+    <t>Correct item is added</t>
+  </si>
+  <si>
+    <t>Verify add product different sort 
+order</t>
+  </si>
+  <si>
+    <t>Check add product different sort order</t>
+  </si>
+  <si>
+    <t>Cart remains correct</t>
+  </si>
+  <si>
+    <t>Verify refresh after add prodcut</t>
+  </si>
+  <si>
+    <t>Check refresh after add product</t>
+  </si>
+  <si>
+    <t>Cart remains correct items after refresh</t>
+  </si>
+  <si>
+    <t>Verify navigate away and return</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check navigate away and return </t>
+  </si>
+  <si>
+    <t>Cart remains correct items after navigate</t>
   </si>
 </sst>
 </file>
@@ -826,7 +1042,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -839,6 +1055,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2053,27 +2275,117 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A14EB0E-C9F5-446A-AC3A-7113DB3CBAFB}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5D70B4-31AF-425E-B314-058EC48D351F}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3CD1F3-4388-420E-9DCC-7F29F14CF0F2}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -2915,54 +3227,901 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0FA298D-6FF1-477B-80FD-74269FD9667C}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="C4:K17"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="2"/>
+    <col min="4" max="4" width="36.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="35.140625" style="2" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="32.5703125" style="2" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="2"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="3:11" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>244</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>248</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>245</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>249</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>251</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>253</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>257</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>255</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>258</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>259</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C13" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>261</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="3" t="s">
+        <v>263</v>
+      </c>
+      <c r="I13" s="3" t="s">
+        <v>264</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>265</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="I14" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>268</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>271</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C16" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>272</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="3:3" x14ac:dyDescent="0.25">
+      <c r="C17" s="2" t="s">
+        <v>61</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DD0F7FEB-1737-4525-899E-F8366C8D679B}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <dimension ref="C4:K14"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="35.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>277</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>293</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>297</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>298</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>299</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>300</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>301</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CECB10C-B31C-4A0D-828C-7D22B0AF58A3}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C362B257-AC70-4114-A9A5-AD73A9E9518C}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DC3CD6E-A0D9-4EF9-BACA-550C85FF5139}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01FDDB4-9F0C-42D6-81C8-5BE55845344D}">
-  <dimension ref="A1"/>
+  <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
write test case remove item from cart
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8212CC8-44D8-4AAC-8724-696871B4309B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97DF837-7D0C-410D-A32B-8E2070F05D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="777" uniqueCount="306">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="338">
   <si>
     <t>Test ID</t>
   </si>
@@ -988,6 +988,102 @@
   </si>
   <si>
     <t>Cart remains correct items after navigate</t>
+  </si>
+  <si>
+    <t>Verify remove item from product page</t>
+  </si>
+  <si>
+    <t>Check remove item from prodcut page</t>
+  </si>
+  <si>
+    <t>Product will remove from the cart</t>
+  </si>
+  <si>
+    <t>Produt is remove from the cart</t>
+  </si>
+  <si>
+    <t>Verify remove item from details page</t>
+  </si>
+  <si>
+    <t>Check remove item from details page</t>
+  </si>
+  <si>
+    <t>Verify remove item from cart page</t>
+  </si>
+  <si>
+    <t>Check remove item from cart page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Check remove one item from multiple item </t>
+  </si>
+  <si>
+    <t>Selected product will remove from the cart</t>
+  </si>
+  <si>
+    <t>Selected product is remove from the cart</t>
+  </si>
+  <si>
+    <t>Verify cart badge after remove item</t>
+  </si>
+  <si>
+    <t>Check cart badge after remove item</t>
+  </si>
+  <si>
+    <t>Cart badge item decreases correctly</t>
+  </si>
+  <si>
+    <t>Verify remove last item</t>
+  </si>
+  <si>
+    <t>Verify remove one item from multiple items</t>
+  </si>
+  <si>
+    <t>Check remove last item from cart</t>
+  </si>
+  <si>
+    <t>Cart badge become empty</t>
+  </si>
+  <si>
+    <t>Verify remove all products</t>
+  </si>
+  <si>
+    <t>Check remove all products</t>
+  </si>
+  <si>
+    <t>Cart become empty</t>
+  </si>
+  <si>
+    <t>Verify add item after removing</t>
+  </si>
+  <si>
+    <t>Check add item after removing</t>
+  </si>
+  <si>
+    <t>Product can be added aging</t>
+  </si>
+  <si>
+    <t>Product added aging</t>
+  </si>
+  <si>
+    <t>Verify remove item after page refresh</t>
+  </si>
+  <si>
+    <t>Check remove item after page refresh</t>
+  </si>
+  <si>
+    <t>product remove successfully</t>
+  </si>
+  <si>
+    <t>Verify multiple remove actions</t>
+  </si>
+  <si>
+    <t>Check multiple remove actions</t>
+  </si>
+  <si>
+    <t>Product remove successfully</t>
+  </si>
+  <si>
+    <t>Cart has no inconsistent state</t>
   </si>
 </sst>
 </file>
@@ -3972,10 +4068,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5CECB10C-B31C-4A0D-828C-7D22B0AF58A3}">
-  <dimension ref="C4:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C4:K14"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="38.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="39" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="38.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="37" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
@@ -4004,7 +4110,298 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>307</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>321</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>315</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>317</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>318</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>319</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>320</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>322</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>323</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>324</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>325</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>326</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>327</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>328</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>329</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>331</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>332</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>336</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>333</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>334</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>335</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>337</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>155</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test cases for cart page
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97DF837-7D0C-410D-A32B-8E2070F05D07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15F6FA7-00BD-4599-9AC4-AA476E0EA92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="338">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="390">
   <si>
     <t>Test ID</t>
   </si>
@@ -1084,6 +1084,166 @@
   </si>
   <si>
     <t>Cart has no inconsistent state</t>
+  </si>
+  <si>
+    <t>Verify cart with one product</t>
+  </si>
+  <si>
+    <t>Check cart with one product</t>
+  </si>
+  <si>
+    <t>Must be Login</t>
+  </si>
+  <si>
+    <t>Display added product</t>
+  </si>
+  <si>
+    <t>Verify cart with mulitple product</t>
+  </si>
+  <si>
+    <t>Check cart with multiple products</t>
+  </si>
+  <si>
+    <t>Display all added products</t>
+  </si>
+  <si>
+    <t>Verify cart without product</t>
+  </si>
+  <si>
+    <t>Check cart page witout product</t>
+  </si>
+  <si>
+    <t>Empty cart page displays correctly</t>
+  </si>
+  <si>
+    <t>Verify cart item name</t>
+  </si>
+  <si>
+    <t>Check cart item name</t>
+  </si>
+  <si>
+    <t>Item correct name in the cart</t>
+  </si>
+  <si>
+    <t>Verify cart item price</t>
+  </si>
+  <si>
+    <t>Check cart item price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Item correct price in the cart </t>
+  </si>
+  <si>
+    <t>Verify cart item description</t>
+  </si>
+  <si>
+    <t>Check cart item description</t>
+  </si>
+  <si>
+    <t>Correct description display in the cart</t>
+  </si>
+  <si>
+    <t>Verify the cart quentity</t>
+  </si>
+  <si>
+    <t>Check the cart item quentity</t>
+  </si>
+  <si>
+    <t>Display will actual quentity</t>
+  </si>
+  <si>
+    <t>Actual quentity is display in the cart</t>
+  </si>
+  <si>
+    <t>Verify cart item image</t>
+  </si>
+  <si>
+    <t>Check the cart item image</t>
+  </si>
+  <si>
+    <t>Item image display in the cart page</t>
+  </si>
+  <si>
+    <t>Item image not show in cart page</t>
+  </si>
+  <si>
+    <t>Verify continue shopping button</t>
+  </si>
+  <si>
+    <t>Check the continue shopping button</t>
+  </si>
+  <si>
+    <t>User return to the product page</t>
+  </si>
+  <si>
+    <t>Verify remove item from cart</t>
+  </si>
+  <si>
+    <t>Check remove item from cart</t>
+  </si>
+  <si>
+    <t>Selected item remove</t>
+  </si>
+  <si>
+    <t>Verify checkout button is visible</t>
+  </si>
+  <si>
+    <t>Check checkout button visible</t>
+  </si>
+  <si>
+    <t>User proceeds to checkout by clicking
+ checkout button</t>
+  </si>
+  <si>
+    <t>Verify checkout with items</t>
+  </si>
+  <si>
+    <t>Check checkout with item</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User proceeds to checkout </t>
+  </si>
+  <si>
+    <t>Verify checkout empty cart</t>
+  </si>
+  <si>
+    <t>Check checkout empty cart</t>
+  </si>
+  <si>
+    <t>User proceed to checkout with
+ empty cart</t>
+  </si>
+  <si>
+    <t>Verify refresh to the cart page</t>
+  </si>
+  <si>
+    <t>Check refresh cart page</t>
+  </si>
+  <si>
+    <t>User not proceed to checkout with
+empty cart</t>
+  </si>
+  <si>
+    <t>Cart data behaves consistently</t>
+  </si>
+  <si>
+    <t>Verify browser back from cart</t>
+  </si>
+  <si>
+    <t>Check browser back for navigate</t>
+  </si>
+  <si>
+    <t>Navigation work correctly</t>
+  </si>
+  <si>
+    <t>Verify cart badge matches with 
+cart items</t>
+  </si>
+  <si>
+    <t>Check cart badge with cart items</t>
+  </si>
+  <si>
+    <t>Cart badge and cart quentity are same</t>
   </si>
 </sst>
 </file>
@@ -1138,7 +1298,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1158,6 +1318,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4408,10 +4571,19 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C362B257-AC70-4114-A9A5-AD73A9E9518C}">
-  <dimension ref="C4:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C4:K20"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="29.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="34.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
@@ -4440,7 +4612,472 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>338</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>339</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>341</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>343</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>344</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>345</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>346</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>347</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>352</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>354</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>360</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C12" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>361</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>362</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>363</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>365</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>366</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="I13" s="1" t="s">
+        <v>367</v>
+      </c>
+      <c r="J13" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C14" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" s="6" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C15" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>371</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>372</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="I15" s="8" t="s">
+        <v>373</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>374</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>375</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="I16" s="1" t="s">
+        <v>376</v>
+      </c>
+      <c r="J16" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C17" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>377</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>378</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="I17" s="7" t="s">
+        <v>379</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>380</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>381</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="I18" s="1" t="s">
+        <v>383</v>
+      </c>
+      <c r="J18" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>384</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>385</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>386</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="20" spans="3:11" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C20" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>388</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="I20" s="1" t="s">
+        <v>389</v>
+      </c>
+      <c r="J20" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write test case for checkout page
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E15F6FA7-00BD-4599-9AC4-AA476E0EA92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013CA937-4C54-46B8-8FF0-76E47DAFA7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="3" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1011" uniqueCount="390">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="432">
   <si>
     <t>Test ID</t>
   </si>
@@ -1244,6 +1244,150 @@
   </si>
   <si>
     <t>Cart badge and cart quentity are same</t>
+  </si>
+  <si>
+    <t>Verify checkout page</t>
+  </si>
+  <si>
+    <t>Check the checkout page</t>
+  </si>
+  <si>
+    <t>Display the customer information form</t>
+  </si>
+  <si>
+    <t>Verify with valid data</t>
+  </si>
+  <si>
+    <t>Check checkout form with valid data</t>
+  </si>
+  <si>
+    <t>Navigae to the checkout overview page</t>
+  </si>
+  <si>
+    <t>FirstName: Abc
+L:astName: xyz
+Zip Code: 723482</t>
+  </si>
+  <si>
+    <t>Verify with invalid data</t>
+  </si>
+  <si>
+    <t>Check checkout form with invalid data</t>
+  </si>
+  <si>
+    <t>FirstName: 2834
+L:astName: 7654
+Zip Code: aksdl</t>
+  </si>
+  <si>
+    <t>Not Navigae to the checkout overview page</t>
+  </si>
+  <si>
+    <t>Criticle</t>
+  </si>
+  <si>
+    <t>Verify with a missing field</t>
+  </si>
+  <si>
+    <t>FirstName: Abc
+L:astName: 
+Zip Code: 12347</t>
+  </si>
+  <si>
+    <t>Validation error message will display</t>
+  </si>
+  <si>
+    <t>Verify with all field missing</t>
+  </si>
+  <si>
+    <t>Check checkout form with a missing field</t>
+  </si>
+  <si>
+    <t>Check checkout form with all missing field</t>
+  </si>
+  <si>
+    <t>empty data</t>
+  </si>
+  <si>
+    <t>Verify numeric name field</t>
+  </si>
+  <si>
+    <t>Check checkout form with numaric name</t>
+  </si>
+  <si>
+    <t>FirstName: 3849
+L:astName: 12421
+Zip Code: 12347</t>
+  </si>
+  <si>
+    <t>Validation behaves correctly</t>
+  </si>
+  <si>
+    <t>Verify with alphabetic zip code</t>
+  </si>
+  <si>
+    <t>Check with alphabetic zip code</t>
+  </si>
+  <si>
+    <t>FirstName: adkll
+L:astName: xyz
+Zip Code: wiurwe</t>
+  </si>
+  <si>
+    <t>Verify name with special Character</t>
+  </si>
+  <si>
+    <t>Check name with special character</t>
+  </si>
+  <si>
+    <t>FirstName: &amp;^%$
+L:astName: @#$
+Zip Code: wiurwe</t>
+  </si>
+  <si>
+    <t>Input hand Safely</t>
+  </si>
+  <si>
+    <t>Verify with special character zip code</t>
+  </si>
+  <si>
+    <t>Check special charcter in zip code</t>
+  </si>
+  <si>
+    <t>FirstName: adcd
+L:astName: sklskd
+Zip Code: &amp;%$#</t>
+  </si>
+  <si>
+    <t>Verify submit with Enter key</t>
+  </si>
+  <si>
+    <t>Check submit with Enter key</t>
+  </si>
+  <si>
+    <t>FirstName: adcd
+L:astName: sklskd
+Zip Code: 2233</t>
+  </si>
+  <si>
+    <t>Form submit successfully with Enter key</t>
+  </si>
+  <si>
+    <t>Check cancel checkout page</t>
+  </si>
+  <si>
+    <t>Verify Cancel Checkout</t>
+  </si>
+  <si>
+    <t>FirstName: adcd
+L:astName: sklskd
+Zip Code: 2234</t>
+  </si>
+  <si>
+    <t>After cancel return to Cart page</t>
+  </si>
+  <si>
+    <t>After cancel retur to product page</t>
   </si>
 </sst>
 </file>
@@ -5084,10 +5228,20 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5DC3CD6E-A0D9-4EF9-BACA-550C85FF5139}">
-  <dimension ref="C4:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C4:K15"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="34.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="17" style="1" customWidth="1"/>
+    <col min="8" max="8" width="40.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="36" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
@@ -5116,7 +5270,327 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>390</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>391</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>392</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>393</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>394</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>396</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C7" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>397</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>398</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>399</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>400</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>401</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C8" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>402</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>406</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>403</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>405</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>407</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>404</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="C10" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>409</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>410</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>411</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" s="2" customFormat="1" ht="47.25" x14ac:dyDescent="0.25">
+      <c r="C11" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>413</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>414</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>415</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>412</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="C12" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>416</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>417</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>418</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" ht="63" x14ac:dyDescent="0.25">
+      <c r="C13" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>421</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>422</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>419</v>
+      </c>
+      <c r="I13" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="C14" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>423</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>424</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>425</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>426</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" s="2" customFormat="1" ht="63" x14ac:dyDescent="0.25">
+      <c r="C15" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>428</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>427</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>429</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>430</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="2" t="s">
+        <v>188</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
write tesct case for checkout overview page
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{013CA937-4C54-46B8-8FF0-76E47DAFA7DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FB073F-F198-4BC9-AA64-469F2497EE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -20,11 +20,12 @@
     <sheet name="Add to Cart" sheetId="5" r:id="rId5"/>
     <sheet name="Remove From Cart" sheetId="6" r:id="rId6"/>
     <sheet name="Cart" sheetId="7" r:id="rId7"/>
-    <sheet name="Chaeckout page" sheetId="8" r:id="rId8"/>
-    <sheet name="Hamburger Menu" sheetId="9" r:id="rId9"/>
-    <sheet name="Logout" sheetId="10" r:id="rId10"/>
-    <sheet name="URL and Session" sheetId="11" r:id="rId11"/>
-    <sheet name="Browser" sheetId="12" r:id="rId12"/>
+    <sheet name="Chaeckout Form" sheetId="8" r:id="rId8"/>
+    <sheet name="Checkout Overview" sheetId="13" r:id="rId9"/>
+    <sheet name="Hamburger Menu" sheetId="9" r:id="rId10"/>
+    <sheet name="Logout" sheetId="10" r:id="rId11"/>
+    <sheet name="URL and Session" sheetId="11" r:id="rId12"/>
+    <sheet name="Browser" sheetId="12" r:id="rId13"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1110" uniqueCount="432">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1254" uniqueCount="478">
   <si>
     <t>Test ID</t>
   </si>
@@ -1388,13 +1389,152 @@
   </si>
   <si>
     <t>After cancel retur to product page</t>
+  </si>
+  <si>
+    <t>Verify with valid information</t>
+  </si>
+  <si>
+    <t>Check with valid information</t>
+  </si>
+  <si>
+    <t>Checkout overview page is open</t>
+  </si>
+  <si>
+    <t>Overview page is opens</t>
+  </si>
+  <si>
+    <t>Verify all selected products</t>
+  </si>
+  <si>
+    <t>Check all selected product</t>
+  </si>
+  <si>
+    <t>Correct products are displayed</t>
+  </si>
+  <si>
+    <t>Verify product name</t>
+  </si>
+  <si>
+    <t>Check the product name</t>
+  </si>
+  <si>
+    <t>Product name match with cart</t>
+  </si>
+  <si>
+    <t>Check product price</t>
+  </si>
+  <si>
+    <t>Product price match with cart</t>
+  </si>
+  <si>
+    <t>Verify product quentity</t>
+  </si>
+  <si>
+    <t>Check product quentity</t>
+  </si>
+  <si>
+    <t>Product quentity match with cart</t>
+  </si>
+  <si>
+    <t>Verify item subtotal</t>
+  </si>
+  <si>
+    <t>Check item subtotal</t>
+  </si>
+  <si>
+    <t>Items price calculate is correct</t>
+  </si>
+  <si>
+    <t>Critical</t>
+  </si>
+  <si>
+    <t>Check subtotal tax</t>
+  </si>
+  <si>
+    <t>Tax calculate is correct</t>
+  </si>
+  <si>
+    <t>Verify Tax amount</t>
+  </si>
+  <si>
+    <t>Verify grand total total + tax</t>
+  </si>
+  <si>
+    <t>Check total amount item price
+total + tax</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Grand total amount is exact </t>
+  </si>
+  <si>
+    <t>Verify payment information</t>
+  </si>
+  <si>
+    <t>Check the payment information</t>
+  </si>
+  <si>
+    <t>Display the correct payment information</t>
+  </si>
+  <si>
+    <t>Verify Shipping information</t>
+  </si>
+  <si>
+    <t>Check the shiping information</t>
+  </si>
+  <si>
+    <t>Display the correct shipping information</t>
+  </si>
+  <si>
+    <t>Verify checkout cancle</t>
+  </si>
+  <si>
+    <t>Check checkout cancle</t>
+  </si>
+  <si>
+    <t>User returns appropriately</t>
+  </si>
+  <si>
+    <t>Verify finish order</t>
+  </si>
+  <si>
+    <t>Check the finish order</t>
+  </si>
+  <si>
+    <t>Order compleate successfully</t>
+  </si>
+  <si>
+    <t>Verify refresh checkout overview page</t>
+  </si>
+  <si>
+    <t>Check refresh overview page</t>
+  </si>
+  <si>
+    <t>No change after refresh</t>
+  </si>
+  <si>
+    <t>Verfy total amount for one items</t>
+  </si>
+  <si>
+    <t>Check total amout for one item</t>
+  </si>
+  <si>
+    <t>Calculation correctly</t>
+  </si>
+  <si>
+    <t>Verify decimal price calculations</t>
+  </si>
+  <si>
+    <t>Check decimal price calculation</t>
+  </si>
+  <si>
+    <t>Correctly calculate decimal price</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1421,6 +1561,13 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1442,7 +1589,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1465,6 +1612,16 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2677,6 +2834,45 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01FDDB4-9F0C-42D6-81C8-5BE55845344D}">
+  <dimension ref="C4:K4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="C4" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="I4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>7</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A14EB0E-C9F5-446A-AC3A-7113DB3CBAFB}">
   <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2715,7 +2911,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C5D70B4-31AF-425E-B314-058EC48D351F}">
   <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2754,7 +2950,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C3CD1F3-4388-420E-9DCC-7F29F14CF0F2}">
   <dimension ref="C4:K4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -5596,11 +5792,21 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01FDDB4-9F0C-42D6-81C8-5BE55845344D}">
-  <dimension ref="C4:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6E9B20-A4F8-48FD-BAAA-C6C6F1645CFC}">
+  <dimension ref="C4:K19"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="9"/>
+    <col min="4" max="4" width="37.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.42578125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="9" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="39.28515625" style="9" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.7109375" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="9.140625" style="9"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
@@ -5629,7 +5835,443 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="9" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>432</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>433</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="9" t="s">
+        <v>434</v>
+      </c>
+      <c r="I5" s="9" t="s">
+        <v>435</v>
+      </c>
+      <c r="J5" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K5" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>436</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>437</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="I6" s="9" t="s">
+        <v>438</v>
+      </c>
+      <c r="J6" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>439</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>440</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>441</v>
+      </c>
+      <c r="J7" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K7" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="9" t="s">
+        <v>172</v>
+      </c>
+      <c r="E8" s="9" t="s">
+        <v>442</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="I8" s="9" t="s">
+        <v>443</v>
+      </c>
+      <c r="J8" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="9" t="s">
+        <v>444</v>
+      </c>
+      <c r="E9" s="9" t="s">
+        <v>445</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="I9" s="9" t="s">
+        <v>446</v>
+      </c>
+      <c r="J9" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="9" t="s">
+        <v>447</v>
+      </c>
+      <c r="E10" s="9" t="s">
+        <v>448</v>
+      </c>
+      <c r="F10" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>449</v>
+      </c>
+      <c r="J10" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="9" t="s">
+        <v>453</v>
+      </c>
+      <c r="E11" s="9" t="s">
+        <v>451</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="I11" s="9" t="s">
+        <v>452</v>
+      </c>
+      <c r="J11" s="9" t="s">
+        <v>450</v>
+      </c>
+      <c r="K11" s="9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" s="11" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="C12" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>454</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>455</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="I12" s="11" t="s">
+        <v>456</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" s="9" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>457</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>458</v>
+      </c>
+      <c r="F13" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="I13" s="9" t="s">
+        <v>459</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C14" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="D14" s="9" t="s">
+        <v>460</v>
+      </c>
+      <c r="E14" s="9" t="s">
+        <v>461</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H14" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="I14" s="9" t="s">
+        <v>462</v>
+      </c>
+      <c r="J14" s="10" t="s">
+        <v>450</v>
+      </c>
+      <c r="K14" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C15" s="9" t="s">
+        <v>59</v>
+      </c>
+      <c r="D15" s="9" t="s">
+        <v>463</v>
+      </c>
+      <c r="E15" s="9" t="s">
+        <v>464</v>
+      </c>
+      <c r="F15" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G15" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H15" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="I15" s="9" t="s">
+        <v>465</v>
+      </c>
+      <c r="J15" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K15" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="16" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C16" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D16" s="9" t="s">
+        <v>466</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>467</v>
+      </c>
+      <c r="F16" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H16" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="I16" s="9" t="s">
+        <v>468</v>
+      </c>
+      <c r="J16" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K16" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C17" s="9" t="s">
+        <v>61</v>
+      </c>
+      <c r="D17" s="9" t="s">
+        <v>469</v>
+      </c>
+      <c r="E17" s="9" t="s">
+        <v>470</v>
+      </c>
+      <c r="F17" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H17" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="I17" s="9" t="s">
+        <v>471</v>
+      </c>
+      <c r="J17" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K17" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="18" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C18" s="9" t="s">
+        <v>62</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>472</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>473</v>
+      </c>
+      <c r="F18" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H18" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="I18" s="9" t="s">
+        <v>474</v>
+      </c>
+      <c r="J18" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K18" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C19" s="9" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="9" t="s">
+        <v>475</v>
+      </c>
+      <c r="E19" s="9" t="s">
+        <v>476</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H19" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="I19" s="9" t="s">
+        <v>477</v>
+      </c>
+      <c r="J19" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K19" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
write hamburger menu test cases
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FB073F-F198-4BC9-AA64-469F2497EE4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2FC9D0-17AB-4833-8A8E-62E8787A1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1254" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="526">
   <si>
     <t>Test ID</t>
   </si>
@@ -1528,6 +1528,150 @@
   </si>
   <si>
     <t>Correctly calculate decimal price</t>
+  </si>
+  <si>
+    <t>Verify Compleate order</t>
+  </si>
+  <si>
+    <t>Check compleate order</t>
+  </si>
+  <si>
+    <t>Redirect to confirm page</t>
+  </si>
+  <si>
+    <t>Verify order successful message</t>
+  </si>
+  <si>
+    <t>Check order successful message</t>
+  </si>
+  <si>
+    <t>Order confirm message visible</t>
+  </si>
+  <si>
+    <t>Verify order success image</t>
+  </si>
+  <si>
+    <t>Check order success image</t>
+  </si>
+  <si>
+    <t>Order successful image is visible</t>
+  </si>
+  <si>
+    <t>Verfiy Back Home button</t>
+  </si>
+  <si>
+    <t>Check back to home button</t>
+  </si>
+  <si>
+    <t>Redirect to home page</t>
+  </si>
+  <si>
+    <t>Verfiy cart after order complite</t>
+  </si>
+  <si>
+    <t>Check cart after order</t>
+  </si>
+  <si>
+    <t>Cart data is clear after order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify refresh </t>
+  </si>
+  <si>
+    <t>Check refresh</t>
+  </si>
+  <si>
+    <t>Application handle refresh safely</t>
+  </si>
+  <si>
+    <t>Verify open Menu</t>
+  </si>
+  <si>
+    <t>Check to open menu</t>
+  </si>
+  <si>
+    <t>Menu will be open</t>
+  </si>
+  <si>
+    <t>Menu is open</t>
+  </si>
+  <si>
+    <t xml:space="preserve">High </t>
+  </si>
+  <si>
+    <t>Verify Close Menu</t>
+  </si>
+  <si>
+    <t>Check to close menu</t>
+  </si>
+  <si>
+    <t>Menu will be close</t>
+  </si>
+  <si>
+    <t>Menu is close</t>
+  </si>
+  <si>
+    <t>Verify all items options</t>
+  </si>
+  <si>
+    <t>Check to all options</t>
+  </si>
+  <si>
+    <t>All menu items visible</t>
+  </si>
+  <si>
+    <t>Verify about option</t>
+  </si>
+  <si>
+    <t>Check about option visible</t>
+  </si>
+  <si>
+    <t>About option is visible</t>
+  </si>
+  <si>
+    <t>Verify click about option</t>
+  </si>
+  <si>
+    <t>Check to click about option</t>
+  </si>
+  <si>
+    <t>User navigate to correctly</t>
+  </si>
+  <si>
+    <t>Verify logout option</t>
+  </si>
+  <si>
+    <t>Check to logout option visible</t>
+  </si>
+  <si>
+    <t>Logout option is visible</t>
+  </si>
+  <si>
+    <t>Verify Click to Logout</t>
+  </si>
+  <si>
+    <t>Check click to logout</t>
+  </si>
+  <si>
+    <t>User Loged out</t>
+  </si>
+  <si>
+    <t>Verify reset app sate</t>
+  </si>
+  <si>
+    <t>Check reset app sate is visible</t>
+  </si>
+  <si>
+    <t>Reset app state is visible</t>
+  </si>
+  <si>
+    <t>Verify App State with cart items</t>
+  </si>
+  <si>
+    <t>Check app sate with cart items</t>
+  </si>
+  <si>
+    <t>Cart is clear</t>
   </si>
 </sst>
 </file>
@@ -2835,8 +2979,15 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B01FDDB4-9F0C-42D6-81C8-5BE55845344D}">
-  <dimension ref="C4:K4"/>
+  <dimension ref="C4:K13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="23.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
@@ -2867,7 +3018,269 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" t="s">
+        <v>496</v>
+      </c>
+      <c r="E5" t="s">
+        <v>497</v>
+      </c>
+      <c r="F5" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>498</v>
+      </c>
+      <c r="I5" t="s">
+        <v>499</v>
+      </c>
+      <c r="J5" t="s">
+        <v>500</v>
+      </c>
+      <c r="K5" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" t="s">
+        <v>501</v>
+      </c>
+      <c r="E6" t="s">
+        <v>502</v>
+      </c>
+      <c r="F6" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>503</v>
+      </c>
+      <c r="I6" t="s">
+        <v>504</v>
+      </c>
+      <c r="J6" t="s">
+        <v>500</v>
+      </c>
+      <c r="K6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" t="s">
+        <v>505</v>
+      </c>
+      <c r="E7" t="s">
+        <v>506</v>
+      </c>
+      <c r="F7" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" t="s">
+        <v>507</v>
+      </c>
+      <c r="I7" t="s">
+        <v>507</v>
+      </c>
+      <c r="J7" t="s">
+        <v>500</v>
+      </c>
+      <c r="K7" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>508</v>
+      </c>
+      <c r="E8" t="s">
+        <v>509</v>
+      </c>
+      <c r="F8" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" t="s">
+        <v>510</v>
+      </c>
+      <c r="I8" t="s">
+        <v>510</v>
+      </c>
+      <c r="J8" t="s">
+        <v>500</v>
+      </c>
+      <c r="K8" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" t="s">
+        <v>511</v>
+      </c>
+      <c r="E9" t="s">
+        <v>512</v>
+      </c>
+      <c r="F9" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" t="s">
+        <v>513</v>
+      </c>
+      <c r="I9" t="s">
+        <v>513</v>
+      </c>
+      <c r="J9" t="s">
+        <v>500</v>
+      </c>
+      <c r="K9" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" t="s">
+        <v>514</v>
+      </c>
+      <c r="E10" t="s">
+        <v>515</v>
+      </c>
+      <c r="F10" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" t="s">
+        <v>12</v>
+      </c>
+      <c r="H10" t="s">
+        <v>516</v>
+      </c>
+      <c r="I10" t="s">
+        <v>516</v>
+      </c>
+      <c r="J10" t="s">
+        <v>500</v>
+      </c>
+      <c r="K10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" t="s">
+        <v>517</v>
+      </c>
+      <c r="E11" t="s">
+        <v>518</v>
+      </c>
+      <c r="F11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H11" t="s">
+        <v>519</v>
+      </c>
+      <c r="I11" t="s">
+        <v>519</v>
+      </c>
+      <c r="J11" t="s">
+        <v>500</v>
+      </c>
+      <c r="K11" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="12" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" t="s">
+        <v>520</v>
+      </c>
+      <c r="E12" t="s">
+        <v>521</v>
+      </c>
+      <c r="F12" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" t="s">
+        <v>12</v>
+      </c>
+      <c r="H12" t="s">
+        <v>522</v>
+      </c>
+      <c r="I12" t="s">
+        <v>522</v>
+      </c>
+      <c r="J12" t="s">
+        <v>500</v>
+      </c>
+      <c r="K12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D13" t="s">
+        <v>523</v>
+      </c>
+      <c r="E13" t="s">
+        <v>524</v>
+      </c>
+      <c r="F13" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" t="s">
+        <v>12</v>
+      </c>
+      <c r="H13" t="s">
+        <v>525</v>
+      </c>
+      <c r="I13" t="s">
+        <v>525</v>
+      </c>
+      <c r="J13" t="s">
+        <v>500</v>
+      </c>
+      <c r="K13" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5793,12 +6206,12 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C6E9B20-A4F8-48FD-BAAA-C6C6F1645CFC}">
-  <dimension ref="C4:K19"/>
+  <dimension ref="C4:K25"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="3" width="9.140625" style="9"/>
     <col min="4" max="4" width="37.28515625" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="30.42578125" style="9" customWidth="1"/>
+    <col min="5" max="5" width="31.85546875" style="9" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.140625" style="9" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.5703125" style="9" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="39.28515625" style="9" bestFit="1" customWidth="1"/>
@@ -6270,6 +6683,180 @@
         <v>15</v>
       </c>
     </row>
+    <row r="20" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C20" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>478</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>479</v>
+      </c>
+      <c r="F20" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H20" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="I20" s="9" t="s">
+        <v>480</v>
+      </c>
+      <c r="J20" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K20" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C21" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="D21" s="9" t="s">
+        <v>481</v>
+      </c>
+      <c r="E21" s="9" t="s">
+        <v>482</v>
+      </c>
+      <c r="F21" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H21" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="I21" s="9" t="s">
+        <v>483</v>
+      </c>
+      <c r="J21" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K21" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C22" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>484</v>
+      </c>
+      <c r="E22" s="9" t="s">
+        <v>485</v>
+      </c>
+      <c r="F22" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H22" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>486</v>
+      </c>
+      <c r="J22" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K22" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="23" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C23" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="D23" s="9" t="s">
+        <v>487</v>
+      </c>
+      <c r="E23" s="9" t="s">
+        <v>488</v>
+      </c>
+      <c r="F23" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H23" s="9" t="s">
+        <v>489</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>489</v>
+      </c>
+      <c r="J23" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K23" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="24" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C24" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>490</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>491</v>
+      </c>
+      <c r="F24" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H24" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>492</v>
+      </c>
+      <c r="J24" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K24" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="25" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C25" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="D25" s="9" t="s">
+        <v>493</v>
+      </c>
+      <c r="E25" s="9" t="s">
+        <v>494</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>197</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="H25" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="I25" s="9" t="s">
+        <v>495</v>
+      </c>
+      <c r="J25" s="9" t="s">
+        <v>14</v>
+      </c>
+      <c r="K25" s="10" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
write test case fro logout
</commit_message>
<xml_diff>
--- a/testCases/Test Case for SauceDemo.xlsx
+++ b/testCases/Test Case for SauceDemo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SQA\manualTestingProject\saucedemo\testCases\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB2FC9D0-17AB-4833-8A8E-62E8787A1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FB664FF-A63A-4054-9699-F00FA1148C54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="6" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" firstSheet="8" activeTab="10" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Login_page" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1389" uniqueCount="526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1434" uniqueCount="542">
   <si>
     <t>Test ID</t>
   </si>
@@ -1672,6 +1672,54 @@
   </si>
   <si>
     <t>Cart is clear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verify logout from inventory </t>
+  </si>
+  <si>
+    <t>Check logout from inventory</t>
+  </si>
+  <si>
+    <t>User return to login</t>
+  </si>
+  <si>
+    <t>Verify logout with cart item</t>
+  </si>
+  <si>
+    <t>User logged out successfully</t>
+  </si>
+  <si>
+    <t>Verify Browser back aftrer logout</t>
+  </si>
+  <si>
+    <t>Check logout with cart item</t>
+  </si>
+  <si>
+    <t>Check browser back after logout</t>
+  </si>
+  <si>
+    <t>Protected pages should not expose authenticated session</t>
+  </si>
+  <si>
+    <t>Verify Browser forware after logout</t>
+  </si>
+  <si>
+    <t>Check browser forward after logout</t>
+  </si>
+  <si>
+    <t>Authentication remains enforced</t>
+  </si>
+  <si>
+    <t>Verify login after logout</t>
+  </si>
+  <si>
+    <t>Check login after logout</t>
+  </si>
+  <si>
+    <t>User can log in normally</t>
+  </si>
+  <si>
+    <t>User login normally</t>
   </si>
 </sst>
 </file>
@@ -3287,10 +3335,19 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A14EB0E-C9F5-446A-AC3A-7113DB3CBAFB}">
-  <dimension ref="C4:K4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="C4:K9"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="3" width="9.140625" style="1"/>
+    <col min="4" max="4" width="32.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="32.85546875" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="51.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="1"/>
+  </cols>
   <sheetData>
-    <row r="4" spans="3:11" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="3:11" x14ac:dyDescent="0.25">
       <c r="C4" s="4" t="s">
         <v>0</v>
       </c>
@@ -3319,7 +3376,153 @@
         <v>7</v>
       </c>
     </row>
+    <row r="5" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>526</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>527</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>528</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>529</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>532</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>530</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>531</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>533</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>534</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>535</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>536</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>537</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="9" spans="3:11" x14ac:dyDescent="0.25">
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>538</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>539</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>540</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>541</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>450</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>